<commit_message>
more scaling and notes and csvs
</commit_message>
<xml_diff>
--- a/notes.xlsx
+++ b/notes.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Nextcloud\Old\nn-parallel-c\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E203C739-5FEC-4CA5-8BE4-613345210A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90ADD669-FCEF-4ECD-9E9A-FE24AB57FF5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="notes" sheetId="1" r:id="rId1"/>
+    <sheet name="tau results" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -104,7 +105,7 @@
     <t>v2 backprop</t>
   </si>
   <si>
-    <t>I also went and tested v1's O2 vs O3 optimization, found nothing significant</t>
+    <t>I also went and tested v1's O2 vs O3 optimization, found nothing significant. I think this was a prompt from Danielle asking if O3 maybe did the nested loops better than O2. It was different by ~noise. We will continue doing optimizations in O3 though.</t>
   </si>
 </sst>
 </file>
@@ -140,11 +141,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -425,453 +429,471 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" customWidth="1"/>
+    <col min="1" max="1" width="116.85546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2">
+        <f>'tau results'!B15+'tau results'!B9</f>
+        <v>9473</v>
+      </c>
+      <c r="D7">
+        <f>'tau results'!D21+'tau results'!D27+'tau results'!D33+'tau results'!D39</f>
+        <v>6158</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="2">
+        <f>'tau results'!B10+'tau results'!B16</f>
+        <v>65320</v>
+      </c>
+      <c r="D8" s="2">
+        <f>'tau results'!D22+'tau results'!D28+'tau results'!D34+'tau results'!D40</f>
+        <v>55032.6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <f>'tau results'!B11+'tau results'!B17</f>
+        <v>1021.1</v>
+      </c>
+      <c r="D9">
+        <f>'tau results'!D23+'tau results'!D29+'tau results'!D35+'tau results'!D41</f>
+        <v>996</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3DD2312-E713-4793-8D65-3B47303CDAC5}">
+  <dimension ref="A1:E41"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.140625" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>12124</v>
+      </c>
+      <c r="C3">
+        <v>7903</v>
+      </c>
+      <c r="D3">
+        <f>1-C3/B3</f>
+        <v>0.34815242494226328</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" t="s">
-        <v>6</v>
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1">
+        <v>76550000000</v>
+      </c>
+      <c r="C4" s="1">
+        <v>64520000000</v>
+      </c>
+      <c r="D4">
+        <f>1-C4/B4</f>
+        <v>0.15715218811234488</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5">
-        <v>12124</v>
-      </c>
-      <c r="C5">
-        <v>7903</v>
+        <v>7</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1301000000</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1257000000</v>
       </c>
       <c r="D5">
         <f>1-C5/B5</f>
-        <v>0.34815242494226328</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="1">
-        <v>76550000000</v>
-      </c>
-      <c r="C6" s="1">
-        <v>64520000000</v>
-      </c>
-      <c r="D6">
-        <f>1-C6/B6</f>
-        <v>0.15715218811234488</v>
+        <v>3.382013835511144E-2</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="1">
-        <v>1301000000</v>
-      </c>
-      <c r="C7" s="1">
-        <v>1257000000</v>
-      </c>
-      <c r="D7">
-        <f>1-C7/B7</f>
-        <v>3.382013835511144E-2</v>
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>18</v>
+        <v>1</v>
+      </c>
+      <c r="B9" s="2">
+        <v>3125</v>
+      </c>
+      <c r="C9" s="3">
+        <v>0.25800000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" t="s">
-        <v>5</v>
-      </c>
-      <c r="E10" t="s">
-        <v>8</v>
+      <c r="A10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="2">
+        <v>22310</v>
+      </c>
+      <c r="C10" s="3">
+        <v>0.29099999999999998</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>1</v>
-      </c>
-      <c r="B11" s="2">
-        <v>3125</v>
+        <v>7</v>
+      </c>
+      <c r="B11">
+        <v>482.1</v>
       </c>
       <c r="C11" s="3">
-        <v>0.25800000000000001</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>2</v>
-      </c>
-      <c r="B12" s="2">
-        <v>22310</v>
-      </c>
-      <c r="C12" s="3">
-        <v>0.29099999999999998</v>
+        <v>0.371</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B13">
-        <v>482.1</v>
-      </c>
-      <c r="C13" s="3">
-        <v>0.371</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>1</v>
+      </c>
+      <c r="B15">
+        <v>6348</v>
+      </c>
+      <c r="C15">
+        <v>52.4</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" t="s">
-        <v>5</v>
-      </c>
-      <c r="E16" t="s">
-        <v>8</v>
+      <c r="A16" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16" s="2">
+        <v>43010</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0.56200000000000006</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B17">
-        <v>6348</v>
-      </c>
-      <c r="C17">
-        <v>52.4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>2</v>
-      </c>
-      <c r="B18" s="2">
-        <v>43010</v>
-      </c>
-      <c r="C18" s="3">
-        <v>0.56200000000000006</v>
+        <v>539</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0.41399999999999998</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>7</v>
-      </c>
-      <c r="B19">
-        <v>539</v>
-      </c>
-      <c r="C19" s="3">
-        <v>0.41399999999999998</v>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" t="s">
+        <v>5</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>3534</v>
+      </c>
+      <c r="E21">
+        <v>44.7</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" t="s">
-        <v>5</v>
-      </c>
-      <c r="E22" t="s">
-        <v>8</v>
+      <c r="A22" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" s="2">
+        <v>24840</v>
+      </c>
+      <c r="E22" s="3">
+        <v>0.38500000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D23">
-        <v>3534</v>
-      </c>
-      <c r="E23">
-        <v>44.7</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>2</v>
-      </c>
-      <c r="D24" s="2">
-        <v>24840</v>
-      </c>
-      <c r="E24" s="3">
-        <v>0.38500000000000001</v>
+        <v>492.2</v>
+      </c>
+      <c r="E23" s="3">
+        <v>0.39200000000000002</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25">
-        <v>492.2</v>
-      </c>
-      <c r="E25" s="3">
-        <v>0.39200000000000002</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" t="s">
+        <v>5</v>
+      </c>
+      <c r="E26" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>13</v>
+        <v>1</v>
+      </c>
+      <c r="D27">
+        <v>2238</v>
+      </c>
+      <c r="E27">
+        <v>28.3</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B28" t="s">
-        <v>9</v>
-      </c>
-      <c r="C28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" t="s">
-        <v>5</v>
-      </c>
-      <c r="E28" t="s">
-        <v>8</v>
+      <c r="A28" t="s">
+        <v>2</v>
+      </c>
+      <c r="D28" s="2">
+        <v>28750</v>
+      </c>
+      <c r="E28" s="3">
+        <v>0.44600000000000001</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D29">
-        <v>2238</v>
-      </c>
-      <c r="E29">
-        <v>28.3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>2</v>
-      </c>
-      <c r="D30" s="2">
-        <v>28750</v>
-      </c>
-      <c r="E30" s="3">
-        <v>0.44600000000000001</v>
+        <v>471.7</v>
+      </c>
+      <c r="E29" s="3">
+        <v>0.375</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31">
-        <v>471.7</v>
-      </c>
-      <c r="E31" s="3">
-        <v>0.375</v>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" t="s">
+        <v>5</v>
+      </c>
+      <c r="E32" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>12</v>
+        <v>1</v>
+      </c>
+      <c r="D33">
+        <v>341</v>
+      </c>
+      <c r="E33" s="3">
+        <v>4.2999999999999997E-2</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B34" t="s">
-        <v>9</v>
-      </c>
-      <c r="C34" t="s">
-        <v>10</v>
-      </c>
-      <c r="D34" t="s">
-        <v>5</v>
-      </c>
-      <c r="E34" t="s">
-        <v>8</v>
+      <c r="A34" t="s">
+        <v>2</v>
+      </c>
+      <c r="D34" s="2">
+        <v>1022</v>
+      </c>
+      <c r="E34" s="3">
+        <v>1.6E-2</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D35">
-        <v>341</v>
+        <v>30.2</v>
       </c>
       <c r="E35" s="3">
-        <v>4.2999999999999997E-2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>2</v>
-      </c>
-      <c r="D36" s="2">
-        <v>1022</v>
-      </c>
-      <c r="E36" s="3">
-        <v>1.6E-2</v>
+        <v>2.4E-2</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>7</v>
-      </c>
-      <c r="D37">
-        <v>30.2</v>
-      </c>
-      <c r="E37" s="3">
-        <v>2.4E-2</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B38" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" t="s">
+        <v>5</v>
+      </c>
+      <c r="E38" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>15</v>
+        <v>1</v>
+      </c>
+      <c r="D39">
+        <v>45</v>
+      </c>
+      <c r="E39" s="3">
+        <v>6.0000000000000001E-3</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B40" t="s">
-        <v>9</v>
-      </c>
-      <c r="C40" t="s">
-        <v>10</v>
-      </c>
-      <c r="D40" t="s">
-        <v>5</v>
-      </c>
-      <c r="E40" t="s">
-        <v>8</v>
+      <c r="A40" t="s">
+        <v>2</v>
+      </c>
+      <c r="D40">
+        <v>420.6</v>
+      </c>
+      <c r="E40" s="3">
+        <v>7.0000000000000001E-3</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D41">
-        <v>45</v>
+        <v>1.9</v>
       </c>
       <c r="E41" s="3">
-        <v>6.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>2</v>
-      </c>
-      <c r="D42">
-        <v>420.6</v>
-      </c>
-      <c r="E42" s="3">
-        <v>7.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>7</v>
-      </c>
-      <c r="D43">
-        <v>1.9</v>
-      </c>
-      <c r="E43" s="3">
         <v>2E-3</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B52" t="s">
-        <v>20</v>
-      </c>
-      <c r="C52" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>1</v>
-      </c>
-      <c r="B53" s="2">
-        <f>B17+B11</f>
-        <v>9473</v>
-      </c>
-      <c r="C53">
-        <f>D23+D29+D35+D41</f>
-        <v>6158</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>2</v>
-      </c>
-      <c r="B54" s="2">
-        <f>B12+B18</f>
-        <v>65320</v>
-      </c>
-      <c r="C54" s="2">
-        <f>D24+D30+D36+D42</f>
-        <v>55032.6</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>7</v>
-      </c>
-      <c r="B55">
-        <f>B13+B19</f>
-        <v>1021.1</v>
-      </c>
-      <c r="C55">
-        <f>D25+D31+D37+D43</f>
-        <v>996</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>